<commit_message>
chore: update market data (29513862643)
</commit_message>
<xml_diff>
--- a/output/lootbar_knivesout_market_list.xlsx
+++ b/output/lootbar_knivesout_market_list.xlsx
@@ -1020,10 +1020,10 @@
         </is>
       </c>
       <c r="F9" s="2" t="n">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="G9" s="3" t="n">
-        <v>6396</v>
+        <v>6386</v>
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
@@ -1044,7 +1044,7 @@
         </is>
       </c>
       <c r="L9" s="3" t="n">
-        <v>6504</v>
+        <v>6363</v>
       </c>
       <c r="M9" s="3" t="n">
         <v>1621555</v>
@@ -1053,7 +1053,7 @@
         <v>8919</v>
       </c>
       <c r="O9" s="2" t="n">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="P9" s="2" t="inlineStr">
         <is>
@@ -1084,10 +1084,10 @@
         </is>
       </c>
       <c r="F10" s="2" t="n">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="G10" s="3" t="n">
-        <v>9105</v>
+        <v>9110</v>
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
@@ -1108,7 +1108,7 @@
         </is>
       </c>
       <c r="L10" s="3" t="n">
-        <v>8722</v>
+        <v>8640</v>
       </c>
       <c r="M10" s="3" t="n">
         <v>154006</v>
@@ -1117,7 +1117,7 @@
         <v>17837</v>
       </c>
       <c r="O10" s="2" t="n">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="P10" s="2" t="inlineStr">
         <is>
@@ -1505,7 +1505,7 @@
         <v>1622</v>
       </c>
       <c r="O17" s="2" t="n">
-        <v>546</v>
+        <v>547</v>
       </c>
       <c r="P17" s="2" t="inlineStr">
         <is>
@@ -1559,7 +1559,7 @@
         <v>3243</v>
       </c>
       <c r="O18" s="2" t="n">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="P18" s="2" t="inlineStr">
         <is>
@@ -2077,7 +2077,7 @@
         </is>
       </c>
       <c r="L27" s="3" t="n">
-        <v>1252</v>
+        <v>970</v>
       </c>
       <c r="M27" s="3" t="n">
         <v>1617248</v>
@@ -2396,7 +2396,7 @@
         <v>1622</v>
       </c>
       <c r="O32" s="2" t="n">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="P32" s="2" t="inlineStr">
         <is>
@@ -2491,10 +2491,10 @@
         </is>
       </c>
       <c r="F34" s="2" t="n">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="G34" s="3" t="n">
-        <v>3405</v>
+        <v>3399</v>
       </c>
       <c r="H34" s="2" t="inlineStr">
         <is>
@@ -2524,7 +2524,7 @@
         <v>6486</v>
       </c>
       <c r="O34" s="2" t="n">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="P34" s="2" t="inlineStr">
         <is>
@@ -2588,7 +2588,7 @@
         <v>12972</v>
       </c>
       <c r="O35" s="2" t="n">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="P35" s="2" t="inlineStr">
         <is>
@@ -2739,10 +2739,10 @@
         </is>
       </c>
       <c r="F38" s="2" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="G38" s="3" t="n">
-        <v>3458</v>
+        <v>3289</v>
       </c>
       <c r="H38" s="2" t="inlineStr">
         <is>
@@ -2863,10 +2863,10 @@
         </is>
       </c>
       <c r="F40" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G40" s="3" t="n">
-        <v>3832</v>
+        <v>3243</v>
       </c>
       <c r="H40" s="2" t="inlineStr">
         <is>
@@ -3103,7 +3103,7 @@
         </is>
       </c>
       <c r="D44" s="3" t="n">
-        <v>10589</v>
+        <v>9707</v>
       </c>
       <c r="E44" s="2" t="inlineStr">
         <is>
@@ -3114,7 +3114,7 @@
         <v>40</v>
       </c>
       <c r="G44" s="3" t="n">
-        <v>9669</v>
+        <v>9682</v>
       </c>
       <c r="H44" s="2" t="inlineStr">
         <is>
@@ -3131,16 +3131,16 @@
       </c>
       <c r="K44" s="2" t="inlineStr"/>
       <c r="L44" s="3" t="n">
-        <v>9707</v>
+        <v>10582</v>
       </c>
       <c r="M44" s="3" t="n">
         <v>10683</v>
       </c>
       <c r="N44" s="3" t="n">
-        <v>10808</v>
+        <v>10800</v>
       </c>
       <c r="O44" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="P44" s="2" t="inlineStr">
         <is>
@@ -3258,7 +3258,7 @@
         <v>6486</v>
       </c>
       <c r="O46" s="2" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="P46" s="2" t="inlineStr">
         <is>
@@ -3500,7 +3500,7 @@
         <v>1784</v>
       </c>
       <c r="O50" s="2" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="P50" s="2" t="inlineStr">
         <is>
@@ -3911,7 +3911,7 @@
         </is>
       </c>
       <c r="L57" s="3" t="n">
-        <v>15097</v>
+        <v>14266</v>
       </c>
       <c r="M57" s="3" t="n">
         <v>31406</v>
@@ -3920,7 +3920,7 @@
         <v>15945</v>
       </c>
       <c r="O57" s="2" t="n">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="P57" s="2" t="inlineStr">
         <is>
@@ -3943,18 +3943,18 @@
         </is>
       </c>
       <c r="D58" s="3" t="n">
-        <v>3781</v>
+        <v>5533</v>
       </c>
       <c r="E58" s="2" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="F58" s="2" t="n">
         <v>38</v>
       </c>
       <c r="G58" s="3" t="n">
-        <v>4490</v>
+        <v>4539</v>
       </c>
       <c r="H58" s="2" t="inlineStr">
         <is>
@@ -3975,13 +3975,13 @@
         </is>
       </c>
       <c r="L58" s="3" t="n">
-        <v>5525</v>
+        <v>1649</v>
       </c>
       <c r="M58" s="3" t="n">
         <v>10586</v>
       </c>
       <c r="N58" s="3" t="n">
-        <v>5017</v>
+        <v>5084</v>
       </c>
       <c r="O58" s="2" t="n">
         <v>6</v>
@@ -4039,7 +4039,7 @@
         </is>
       </c>
       <c r="L59" s="3" t="n">
-        <v>4853</v>
+        <v>4368</v>
       </c>
       <c r="M59" s="3" t="n">
         <v>11594</v>
@@ -4048,7 +4048,7 @@
         <v>4728</v>
       </c>
       <c r="O59" s="2" t="n">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="P59" s="2" t="inlineStr">
         <is>
@@ -8347,10 +8347,10 @@
         </is>
       </c>
       <c r="F140" s="2" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="G140" s="3" t="n">
-        <v>427</v>
+        <v>395</v>
       </c>
       <c r="H140" s="2" t="inlineStr">
         <is>
@@ -8530,23 +8530,13 @@
           <t>銃器</t>
         </is>
       </c>
-      <c r="D143" s="3" t="n">
-        <v>2919</v>
-      </c>
-      <c r="E143" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-16</t>
-        </is>
-      </c>
-      <c r="F143" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="G143" s="3" t="n">
-        <v>2919</v>
-      </c>
+      <c r="D143" s="3" t="inlineStr"/>
+      <c r="E143" s="2" t="inlineStr"/>
+      <c r="F143" s="2" t="inlineStr"/>
+      <c r="G143" s="3" t="inlineStr"/>
       <c r="H143" s="2" t="inlineStr">
         <is>
-          <t>※価格トレンドAPI(日次データ)に基づく近似値</t>
+          <t>直近30日間の取引データなし</t>
         </is>
       </c>
       <c r="I143" s="2" t="n">
@@ -8636,7 +8626,7 @@
         <v>4054</v>
       </c>
       <c r="O144" s="2" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="P144" s="2" t="inlineStr">
         <is>
@@ -8929,10 +8919,10 @@
         </is>
       </c>
       <c r="F150" s="2" t="n">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="G150" s="3" t="n">
-        <v>16378</v>
+        <v>16374</v>
       </c>
       <c r="H150" s="2" t="inlineStr">
         <is>
@@ -8962,7 +8952,7 @@
         <v>32431</v>
       </c>
       <c r="O150" s="2" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="P150" s="2" t="inlineStr">
         <is>
@@ -9026,7 +9016,7 @@
         <v>77835</v>
       </c>
       <c r="O151" s="2" t="n">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="P151" s="2" t="inlineStr">
         <is>
@@ -9080,7 +9070,7 @@
         <v>210802</v>
       </c>
       <c r="O152" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="P152" s="2" t="inlineStr">
         <is>
@@ -9388,7 +9378,7 @@
         <v>6486</v>
       </c>
       <c r="O157" s="2" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="P157" s="2" t="inlineStr">
         <is>
@@ -9679,7 +9669,7 @@
         </is>
       </c>
       <c r="L162" s="3" t="n">
-        <v>1947</v>
+        <v>1941</v>
       </c>
       <c r="M162" s="3" t="n">
         <v>30939</v>
@@ -9688,7 +9678,7 @@
         <v>1622</v>
       </c>
       <c r="O162" s="2" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="P162" s="2" t="inlineStr">
         <is>
@@ -9775,7 +9765,7 @@
         </is>
       </c>
       <c r="D164" s="3" t="n">
-        <v>3733</v>
+        <v>3783</v>
       </c>
       <c r="E164" s="2" t="inlineStr">
         <is>
@@ -9786,7 +9776,7 @@
         <v>56</v>
       </c>
       <c r="G164" s="3" t="n">
-        <v>3662</v>
+        <v>3664</v>
       </c>
       <c r="H164" s="2" t="inlineStr">
         <is>
@@ -9816,7 +9806,7 @@
         <v>6486</v>
       </c>
       <c r="O164" s="2" t="n">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="P164" s="2" t="inlineStr">
         <is>
@@ -9880,7 +9870,7 @@
         <v>324</v>
       </c>
       <c r="O165" s="2" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="P165" s="2" t="inlineStr">
         <is>
@@ -10008,7 +9998,7 @@
         <v>1406</v>
       </c>
       <c r="O167" s="2" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="P167" s="2" t="inlineStr">
         <is>
@@ -10532,7 +10522,7 @@
         <v>32431</v>
       </c>
       <c r="O177" s="2" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="P177" s="2" t="inlineStr">
         <is>
@@ -10576,13 +10566,13 @@
         <v>19459</v>
       </c>
       <c r="M178" s="3" t="n">
-        <v>19621</v>
+        <v>33980</v>
       </c>
       <c r="N178" s="3" t="n">
         <v>38917</v>
       </c>
       <c r="O178" s="2" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="P178" s="2" t="inlineStr">
         <is>
@@ -10996,7 +10986,7 @@
         <v>324</v>
       </c>
       <c r="O186" s="2" t="n">
-        <v>367</v>
+        <v>368</v>
       </c>
       <c r="P186" s="2" t="inlineStr">
         <is>
@@ -11436,7 +11426,7 @@
         <v>324</v>
       </c>
       <c r="O194" s="2" t="n">
-        <v>412</v>
+        <v>413</v>
       </c>
       <c r="P194" s="2" t="inlineStr">
         <is>
@@ -11663,7 +11653,7 @@
         <v>16216</v>
       </c>
       <c r="N198" s="3" t="n">
-        <v>582</v>
+        <v>611</v>
       </c>
       <c r="O198" s="2" t="n">
         <v>13</v>
@@ -13402,7 +13392,7 @@
         <v>324</v>
       </c>
       <c r="O229" s="2" t="n">
-        <v>794</v>
+        <v>795</v>
       </c>
       <c r="P229" s="2" t="inlineStr">
         <is>
@@ -13466,7 +13456,7 @@
         <v>324</v>
       </c>
       <c r="O230" s="2" t="n">
-        <v>1121</v>
+        <v>1120</v>
       </c>
       <c r="P230" s="2" t="inlineStr">
         <is>
@@ -13520,7 +13510,7 @@
         <v>1622</v>
       </c>
       <c r="O231" s="2" t="n">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="P231" s="2" t="inlineStr">
         <is>
@@ -14078,12 +14068,18 @@
           <t>Weapon</t>
         </is>
       </c>
-      <c r="L241" s="3" t="inlineStr"/>
-      <c r="M241" s="3" t="inlineStr"/>
+      <c r="L241" s="3" t="n">
+        <v>26383</v>
+      </c>
+      <c r="M241" s="3" t="n">
+        <v>26383</v>
+      </c>
       <c r="N241" s="3" t="n">
         <v>32431</v>
       </c>
-      <c r="O241" s="2" t="inlineStr"/>
+      <c r="O241" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="P241" s="2" t="inlineStr">
         <is>
           <t>2026-07-16</t>
@@ -14137,7 +14133,7 @@
         </is>
       </c>
       <c r="L242" s="3" t="n">
-        <v>40779</v>
+        <v>40193</v>
       </c>
       <c r="M242" s="3" t="n">
         <v>60082</v>
@@ -14146,7 +14142,7 @@
         <v>77835</v>
       </c>
       <c r="O242" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="P242" s="2" t="inlineStr">
         <is>
@@ -14197,7 +14193,7 @@
       </c>
       <c r="K243" s="2" t="inlineStr"/>
       <c r="L243" s="3" t="n">
-        <v>20458</v>
+        <v>20388</v>
       </c>
       <c r="M243" s="3" t="n">
         <v>32431103</v>
@@ -14206,7 +14202,7 @@
         <v>32431</v>
       </c>
       <c r="O243" s="2" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="P243" s="2" t="inlineStr">
         <is>
@@ -14363,7 +14359,7 @@
         </is>
       </c>
       <c r="L246" s="3" t="n">
-        <v>2648</v>
+        <v>2445</v>
       </c>
       <c r="M246" s="3" t="n">
         <v>16216</v>
@@ -14372,7 +14368,7 @@
         <v>3271</v>
       </c>
       <c r="O246" s="2" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="P246" s="2" t="inlineStr">
         <is>
@@ -15029,10 +15025,10 @@
         </is>
       </c>
       <c r="F258" s="2" t="n">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="G258" s="3" t="n">
-        <v>414</v>
+        <v>413</v>
       </c>
       <c r="H258" s="2" t="inlineStr">
         <is>
@@ -15062,7 +15058,7 @@
         <v>649</v>
       </c>
       <c r="O258" s="2" t="n">
-        <v>266</v>
+        <v>361</v>
       </c>
       <c r="P258" s="2" t="inlineStr">
         <is>
@@ -15149,18 +15145,18 @@
         </is>
       </c>
       <c r="D260" s="3" t="n">
-        <v>2726</v>
+        <v>2643</v>
       </c>
       <c r="E260" s="2" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="F260" s="2" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="G260" s="3" t="n">
-        <v>1953</v>
+        <v>2039</v>
       </c>
       <c r="H260" s="2" t="inlineStr">
         <is>
@@ -15181,7 +15177,7 @@
         </is>
       </c>
       <c r="L260" s="3" t="n">
-        <v>2643</v>
+        <v>2659</v>
       </c>
       <c r="M260" s="3" t="n">
         <v>3765</v>
@@ -15190,7 +15186,7 @@
         <v>3243</v>
       </c>
       <c r="O260" s="2" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="P260" s="2" t="inlineStr">
         <is>
@@ -15372,7 +15368,7 @@
         <v>1622</v>
       </c>
       <c r="O263" s="2" t="n">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="P263" s="2" t="inlineStr">
         <is>
@@ -15552,13 +15548,13 @@
         <v>9882</v>
       </c>
       <c r="M266" s="3" t="n">
-        <v>9882</v>
+        <v>12972</v>
       </c>
       <c r="N266" s="3" t="n">
         <v>12972</v>
       </c>
       <c r="O266" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="P266" s="2" t="inlineStr">
         <is>
@@ -16202,7 +16198,7 @@
         <v>1622</v>
       </c>
       <c r="O277" s="2" t="n">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="P277" s="2" t="inlineStr">
         <is>
@@ -16637,7 +16633,7 @@
         </is>
       </c>
       <c r="L285" s="3" t="n">
-        <v>10478</v>
+        <v>10477</v>
       </c>
       <c r="M285" s="3" t="n">
         <v>16216</v>
@@ -16793,7 +16789,7 @@
         </is>
       </c>
       <c r="D288" s="3" t="n">
-        <v>6679</v>
+        <v>7072</v>
       </c>
       <c r="E288" s="2" t="inlineStr">
         <is>
@@ -16801,10 +16797,10 @@
         </is>
       </c>
       <c r="F288" s="2" t="n">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="G288" s="3" t="n">
-        <v>6811</v>
+        <v>6819</v>
       </c>
       <c r="H288" s="2" t="inlineStr">
         <is>
@@ -16821,16 +16817,16 @@
       </c>
       <c r="K288" s="2" t="inlineStr"/>
       <c r="L288" s="3" t="n">
-        <v>7072</v>
+        <v>7266</v>
       </c>
       <c r="M288" s="3" t="n">
         <v>8036</v>
       </c>
       <c r="N288" s="3" t="n">
-        <v>7422</v>
+        <v>7449</v>
       </c>
       <c r="O288" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="P288" s="2" t="inlineStr">
         <is>
@@ -16977,18 +16973,18 @@
         </is>
       </c>
       <c r="D291" s="3" t="n">
-        <v>1951</v>
+        <v>2531</v>
       </c>
       <c r="E291" s="2" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="F291" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G291" s="3" t="n">
-        <v>1951</v>
+        <v>2241</v>
       </c>
       <c r="H291" s="2" t="inlineStr">
         <is>
@@ -17009,7 +17005,7 @@
         </is>
       </c>
       <c r="L291" s="3" t="n">
-        <v>2531</v>
+        <v>3888</v>
       </c>
       <c r="M291" s="3" t="n">
         <v>5189</v>
@@ -17018,7 +17014,7 @@
         <v>3243</v>
       </c>
       <c r="O291" s="2" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="P291" s="2" t="inlineStr">
         <is>
@@ -17049,10 +17045,10 @@
         </is>
       </c>
       <c r="F292" s="2" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="G292" s="3" t="n">
-        <v>4455</v>
+        <v>4503</v>
       </c>
       <c r="H292" s="2" t="inlineStr">
         <is>
@@ -17210,7 +17206,7 @@
         <v>7398</v>
       </c>
       <c r="O294" s="2" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="P294" s="2" t="inlineStr">
         <is>
@@ -17291,11 +17287,11 @@
       </c>
       <c r="E296" s="2" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="F296" s="2" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="G296" s="3" t="n">
         <v>32431</v>
@@ -17328,7 +17324,7 @@
         <v>40539</v>
       </c>
       <c r="O296" s="2" t="n">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="P296" s="2" t="inlineStr">
         <is>
@@ -17392,7 +17388,7 @@
         <v>81078</v>
       </c>
       <c r="O297" s="2" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="P297" s="2" t="inlineStr">
         <is>
@@ -17639,16 +17635,16 @@
         </is>
       </c>
       <c r="L301" s="3" t="n">
-        <v>34215</v>
+        <v>33980</v>
       </c>
       <c r="M301" s="3" t="n">
         <v>34215</v>
       </c>
       <c r="N301" s="3" t="n">
-        <v>17463</v>
+        <v>17067</v>
       </c>
       <c r="O301" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="P301" s="2" t="inlineStr">
         <is>
@@ -17712,7 +17708,7 @@
         <v>2270</v>
       </c>
       <c r="O302" s="2" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="P302" s="2" t="inlineStr">
         <is>
@@ -17743,10 +17739,10 @@
         </is>
       </c>
       <c r="F303" s="2" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="G303" s="3" t="n">
-        <v>4256</v>
+        <v>4298</v>
       </c>
       <c r="H303" s="2" t="inlineStr">
         <is>
@@ -17767,7 +17763,7 @@
         </is>
       </c>
       <c r="L303" s="3" t="n">
-        <v>4391</v>
+        <v>4378</v>
       </c>
       <c r="M303" s="3" t="n">
         <v>16214</v>
@@ -17776,7 +17772,7 @@
         <v>4719</v>
       </c>
       <c r="O303" s="2" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="P303" s="2" t="inlineStr">
         <is>
@@ -18508,7 +18504,7 @@
         <v>32431</v>
       </c>
       <c r="O315" s="2" t="n">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="P315" s="2" t="inlineStr">
         <is>
@@ -18572,7 +18568,7 @@
         <v>77835</v>
       </c>
       <c r="O316" s="2" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="P316" s="2" t="inlineStr">
         <is>
@@ -18626,7 +18622,7 @@
         <v>210802</v>
       </c>
       <c r="O317" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="P317" s="2" t="inlineStr">
         <is>
@@ -18712,23 +18708,13 @@
           <t>お宝 / 宝箱</t>
         </is>
       </c>
-      <c r="D319" s="3" t="n">
-        <v>1378</v>
-      </c>
-      <c r="E319" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-16</t>
-        </is>
-      </c>
-      <c r="F319" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="G319" s="3" t="n">
-        <v>1378</v>
-      </c>
+      <c r="D319" s="3" t="inlineStr"/>
+      <c r="E319" s="2" t="inlineStr"/>
+      <c r="F319" s="2" t="inlineStr"/>
+      <c r="G319" s="3" t="inlineStr"/>
       <c r="H319" s="2" t="inlineStr">
         <is>
-          <t>※価格トレンドAPI(日次データ)に基づく近似値</t>
+          <t>直近30日間の取引データなし</t>
         </is>
       </c>
       <c r="I319" s="2" t="n">
@@ -18937,7 +18923,7 @@
         </is>
       </c>
       <c r="L322" s="3" t="n">
-        <v>522</v>
+        <v>378</v>
       </c>
       <c r="M322" s="3" t="n">
         <v>1067</v>
@@ -19098,7 +19084,7 @@
         <v>17</v>
       </c>
       <c r="G325" s="3" t="n">
-        <v>1801</v>
+        <v>1765</v>
       </c>
       <c r="H325" s="2" t="inlineStr">
         <is>
@@ -19119,7 +19105,7 @@
         </is>
       </c>
       <c r="L325" s="3" t="n">
-        <v>2329</v>
+        <v>2319</v>
       </c>
       <c r="M325" s="3" t="n">
         <v>16105</v>
@@ -19128,7 +19114,7 @@
         <v>2517</v>
       </c>
       <c r="O325" s="2" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="P325" s="2" t="inlineStr">
         <is>
@@ -19247,16 +19233,16 @@
         </is>
       </c>
       <c r="L327" s="3" t="n">
-        <v>3738</v>
+        <v>2912</v>
       </c>
       <c r="M327" s="3" t="n">
         <v>11351</v>
       </c>
       <c r="N327" s="3" t="n">
-        <v>3631</v>
+        <v>3123</v>
       </c>
       <c r="O327" s="2" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="P327" s="2" t="inlineStr">
         <is>
@@ -19279,18 +19265,18 @@
         </is>
       </c>
       <c r="D328" s="3" t="n">
-        <v>22630</v>
+        <v>26211</v>
       </c>
       <c r="E328" s="2" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="F328" s="2" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="G328" s="3" t="n">
-        <v>20821</v>
+        <v>21066</v>
       </c>
       <c r="H328" s="2" t="inlineStr">
         <is>
@@ -19311,16 +19297,16 @@
         </is>
       </c>
       <c r="L328" s="3" t="n">
-        <v>26211</v>
+        <v>24659</v>
       </c>
       <c r="M328" s="3" t="n">
         <v>33422</v>
       </c>
       <c r="N328" s="3" t="n">
-        <v>22090</v>
+        <v>22510</v>
       </c>
       <c r="O328" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="P328" s="2" t="inlineStr">
         <is>
@@ -19375,16 +19361,16 @@
         </is>
       </c>
       <c r="L329" s="3" t="n">
-        <v>6697</v>
+        <v>6668</v>
       </c>
       <c r="M329" s="3" t="n">
         <v>9329</v>
       </c>
       <c r="N329" s="3" t="n">
-        <v>8035</v>
+        <v>7993</v>
       </c>
       <c r="O329" s="2" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="P329" s="2" t="inlineStr">
         <is>
@@ -19439,7 +19425,7 @@
         </is>
       </c>
       <c r="L330" s="3" t="n">
-        <v>6584</v>
+        <v>6407</v>
       </c>
       <c r="M330" s="3" t="n">
         <v>8873</v>
@@ -19448,7 +19434,7 @@
         <v>6770</v>
       </c>
       <c r="O330" s="2" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="P330" s="2" t="inlineStr">
         <is>
@@ -19535,18 +19521,18 @@
         </is>
       </c>
       <c r="D332" s="3" t="n">
-        <v>1148</v>
+        <v>970</v>
       </c>
       <c r="E332" s="2" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="F332" s="2" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="G332" s="3" t="n">
-        <v>1240</v>
+        <v>1217</v>
       </c>
       <c r="H332" s="2" t="inlineStr">
         <is>
@@ -19567,16 +19553,16 @@
         </is>
       </c>
       <c r="L332" s="3" t="n">
-        <v>970</v>
+        <v>1067</v>
       </c>
       <c r="M332" s="3" t="n">
         <v>16216</v>
       </c>
       <c r="N332" s="3" t="n">
-        <v>1262</v>
+        <v>1164</v>
       </c>
       <c r="O332" s="2" t="n">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="P332" s="2" t="inlineStr">
         <is>
@@ -19759,7 +19745,7 @@
         </is>
       </c>
       <c r="L335" s="3" t="n">
-        <v>1938</v>
+        <v>1936</v>
       </c>
       <c r="M335" s="3" t="n">
         <v>4946</v>
@@ -20143,7 +20129,7 @@
         </is>
       </c>
       <c r="L341" s="3" t="n">
-        <v>608</v>
+        <v>606</v>
       </c>
       <c r="M341" s="3" t="n">
         <v>2450</v>
@@ -20216,7 +20202,7 @@
         <v>478</v>
       </c>
       <c r="O342" s="2" t="n">
-        <v>540</v>
+        <v>530</v>
       </c>
       <c r="P342" s="2" t="inlineStr">
         <is>
@@ -20311,10 +20297,10 @@
         </is>
       </c>
       <c r="F344" s="2" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="G344" s="3" t="n">
-        <v>1841</v>
+        <v>1802</v>
       </c>
       <c r="H344" s="2" t="inlineStr">
         <is>
@@ -20335,7 +20321,7 @@
         </is>
       </c>
       <c r="L344" s="3" t="n">
-        <v>1622</v>
+        <v>1746</v>
       </c>
       <c r="M344" s="3" t="n">
         <v>3882</v>
@@ -20344,7 +20330,7 @@
         <v>3243</v>
       </c>
       <c r="O344" s="2" t="n">
-        <v>13</v>
+        <v>18</v>
       </c>
       <c r="P344" s="2" t="inlineStr">
         <is>
@@ -20408,7 +20394,7 @@
         <v>4054</v>
       </c>
       <c r="O345" s="2" t="n">
-        <v>40</v>
+        <v>46</v>
       </c>
       <c r="P345" s="2" t="inlineStr">
         <is>
@@ -20510,7 +20496,7 @@
         <v>6486</v>
       </c>
       <c r="O347" s="2" t="n">
-        <v>21</v>
+        <v>30</v>
       </c>
       <c r="P347" s="2" t="inlineStr">
         <is>
@@ -20554,12 +20540,18 @@
           <t>Weapon</t>
         </is>
       </c>
-      <c r="L348" s="3" t="inlineStr"/>
-      <c r="M348" s="3" t="inlineStr"/>
+      <c r="L348" s="3" t="n">
+        <v>9729</v>
+      </c>
+      <c r="M348" s="3" t="n">
+        <v>9729</v>
+      </c>
       <c r="N348" s="3" t="n">
         <v>12972</v>
       </c>
-      <c r="O348" s="2" t="inlineStr"/>
+      <c r="O348" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="P348" s="2" t="inlineStr">
         <is>
           <t>2026-07-16</t>
@@ -20701,10 +20693,10 @@
         </is>
       </c>
       <c r="F351" s="2" t="n">
-        <v>16</v>
+        <v>24</v>
       </c>
       <c r="G351" s="3" t="n">
-        <v>16512</v>
+        <v>16503</v>
       </c>
       <c r="H351" s="2" t="inlineStr">
         <is>
@@ -20728,13 +20720,13 @@
         <v>16216</v>
       </c>
       <c r="M351" s="3" t="n">
-        <v>48543</v>
+        <v>32431</v>
       </c>
       <c r="N351" s="3" t="n">
         <v>32431</v>
       </c>
       <c r="O351" s="2" t="n">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="P351" s="2" t="inlineStr">
         <is>
@@ -20916,7 +20908,7 @@
         <v>18161</v>
       </c>
       <c r="O354" s="2" t="n">
-        <v>41</v>
+        <v>50</v>
       </c>
       <c r="P354" s="2" t="inlineStr">
         <is>
@@ -20938,13 +20930,23 @@
           <t>お宝 / 宝箱</t>
         </is>
       </c>
-      <c r="D355" s="3" t="inlineStr"/>
-      <c r="E355" s="2" t="inlineStr"/>
-      <c r="F355" s="2" t="inlineStr"/>
-      <c r="G355" s="3" t="inlineStr"/>
+      <c r="D355" s="3" t="n">
+        <v>9081</v>
+      </c>
+      <c r="E355" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="F355" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G355" s="3" t="n">
+        <v>9081</v>
+      </c>
       <c r="H355" s="2" t="inlineStr">
         <is>
-          <t>直近30日間の取引データなし</t>
+          <t>※価格トレンドAPI(日次データ)に基づく近似値</t>
         </is>
       </c>
       <c r="I355" s="2" t="n">
@@ -20970,7 +20972,7 @@
         <v>18161</v>
       </c>
       <c r="O355" s="2" t="n">
-        <v>28</v>
+        <v>34</v>
       </c>
       <c r="P355" s="2" t="inlineStr">
         <is>

</xml_diff>